<commit_message>
docs(threat-model): add T09/T10, M-007 to M-010 and gap-to-improvement sheet
</commit_message>
<xml_diff>
--- a/threat-model/threat-model.xlsx
+++ b/threat-model/threat-model.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WCGW Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Threats" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mitigation Candidates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvements" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -802,7 +803,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Cualquier cliente HTTP, sin autenticacion de por medio, puede registrar una accion mediante POST /actions indicando un campo "analyst" arbitrario, lo que conduce a la suplantacion de la identidad de un analista y afecta negativamente a la integridad de la bitacora de acciones (ACTIONS).</t>
+          <t>Cualquier cliente HTTP, sin autenticación de por medio, puede registrar una acción mediante POST /actions indicando un campo "analyst" arbitrario, lo que conduce a la suplantación de la identidad de un analista y afecta negativamente a la integridad de la bitácora de acciones (ACTIONS).</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -824,7 +825,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Un cliente HTTP, sin TLS ni validacion de esquema, puede enviar POST /alerts con campos severity/host/ioc arbitrarios, lo que conduce a la alteracion o inyeccion de contenido no autorizado y afecta negativamente a la integridad de los datos de alertas (ALERTS).</t>
+          <t>Un cliente HTTP, sin TLS ni validación de esquema, puede enviar POST /alerts con campos severity/host/ioc arbitrarios, lo que conduce a la alteración o inyección de contenido no autorizado y afecta negativamente a la integridad de los datos de alertas (ALERTS).</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -846,7 +847,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Un analista que registra una accion mediante POST /actions puede negar haberla ejecutado, ya que el campo "analyst" no esta ligado a una sesion autenticada ni firmada, lo que conduce a la imposibilidad de atribuir la accion de forma confiable y afecta negativamente a la trazabilidad del almacen de acciones (ACTIONS) y los logs.</t>
+          <t>Un analista que registra una acción mediante POST /actions puede negar haberla ejecutado, ya que el campo "analyst" no está ligado a una sesión autenticada ni firmada, lo que conduce a la imposibilidad de atribuir la acción de forma confiable y afecta negativamente a la trazabilidad del almacén de acciones (ACTIONS) y los logs.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -868,7 +869,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Un cliente HTTP anonimo puede invocar GET /debug/env sin autenticacion, lo que conduce a la exposicion de todas las variables de entorno del servidor y afecta negativamente a la confidencialidad del host y de la configuracion del backend.</t>
+          <t>Un cliente HTTP anónimo puede invocar GET /debug/env sin autenticación, lo que conduce a la exposición de todas las variables de entorno del servidor y afecta negativamente a la confidencialidad del host y de la configuración del backend.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -890,7 +891,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Un cliente HTTP puede enviar rafagas de POST /alerts o /actions sin limite de tasa contra el servidor de desarrollo de Flask (single-threaded), lo que conduce al crecimiento no acotado de las listas en memoria y a la saturacion del proceso, y afecta negativamente a la disponibilidad de alerts-api/actions-api.</t>
+          <t>Un cliente HTTP puede enviar ráfagas de POST /alerts o /actions sin límite de tasa contra el servidor de desarrollo de Flask (single-threaded), lo que conduce al crecimiento no acotado de las listas en memoria y a la saturación del proceso, y afecta negativamente a la disponibilidad de alerts-api/actions-api.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -912,7 +913,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Un cliente HTTP anonimo, sin modelo de autorizacion, puede ejecutar POST /actions con action=close sobre una alerta CRITICAL, lo que conduce a la ejecucion de una accion privilegiada sin verificacion de rol y afecta negativamente a la integridad del proceso de respuesta a incidentes.</t>
+          <t>Un cliente HTTP anónimo, sin modelo de autorización, puede ejecutar POST /actions con action=close sobre una alerta CRITICAL, lo que conduce a la ejecución de una acción privilegiada sin verificación de rol y afecta negativamente a la integridad del proceso de respuesta a incidentes.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -932,9 +933,21 @@
           <t>T09</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Un atacante con acceso a la red del laboratorio puede conectarse directamente a los puertos 5000/5001 de los microservicios Flask (bind 0.0.0.0), lo que conduce a saltarse el proxy de Nginx y sus controles (logs, headers, hardening) y afecta negativamente a la confidencialidad e integridad de ALERTS y ACTIONS.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Nginx → alerts-api / actions-api (frontera L2)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
@@ -942,9 +955,21 @@
           <t>T10</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Un atacante que provoque una excepción no controlada en un servicio con debug=True puede acceder al debugger interactivo de Werkzeug (cuyo PIN queda escrito en alerts.log), lo que conduce a ejecución de código en el host y afecta negativamente a la confidencialidad, integridad y disponibilidad del servidor.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>alerts-api / actions-api (Proceso) / debugger Werkzeug</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -993,7 +1018,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Autenticacion de analistas (roles/sesion) sobre actions-api y alerts-api -- planificado para Lab 4.</t>
+          <t>Autenticación de analistas (roles/sesión) sobre actions-api y alerts-api — planificado para Lab 4.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1010,7 +1035,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Validacion de esquema de entrada (severity/host/ioc) en alerts-api, mas HTTPS/TLS en Lab 4.</t>
+          <t>Validación de esquema de entrada (severity/host/ioc) en alerts-api, más HTTPS/TLS en Lab 4.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1027,7 +1052,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Vincular cada accion a una sesion autenticada; log de auditoria append-only con hash-chain en actions-api.</t>
+          <t>Vincular cada acción a una sesión autenticada; log de auditoría append-only con hash-chain en actions-api.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1061,7 +1086,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Servir alerts-api/actions-api con un WSGI de produccion (gunicorn) y aplicar limit_req en Nginx para limitar tasa y tamano de payload.</t>
+          <t>Servir alerts-api/actions-api con un WSGI de producción (gunicorn) y aplicar limit_req en Nginx para limitar tasa y tamaño de payload.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1078,7 +1103,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Modelo RBAC (viewer/analyst/admin) con verificacion de autorizacion por tipo de accion en actions-api -- Lab 4.</t>
+          <t>Modelo RBAC (viewer/analyst/admin) con verificación de autorización por tipo de acción en actions-api — Lab 4.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1093,8 +1118,16 @@
           <t>M-007</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>[Implementada en repo] Enlazar alerts-api y actions-api únicamente a 127.0.0.1 y configurar UFW (deny incoming; allow OpenSSH; allow 80/tcp desde LAB_CIDR), de modo que Nginx sea el único punto de entrada.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
@@ -1102,8 +1135,16 @@
           <t>M-008</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>[Implementada en repo] Ejecutar ambos servicios con debug=False y eliminar el endpoint /debug/env (retira el debugger de Werkzeug y la exposición de variables de entorno).</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>T06, T10</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
@@ -1111,8 +1152,16 @@
           <t>M-009</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>[Implementada en repo] Registrar la IP real del cliente (X-Real-IP inyectado por Nginx) como source_ip en cada acción y en los logs de ambos servicios, para correlacionarla con access.log.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
@@ -1120,8 +1169,16 @@
           <t>M-010</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>[Implementada en repo] Hardening de Nginx: server_tokens off, X-Content-Type-Options, X-Frame-Options, Referrer-Policy, autoindex off y denegación de rutas ocultas.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
@@ -1243,4 +1300,324 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3.5546875" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura inicial</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Gap identificado</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Riesgo / Amenaza</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Mejora implementada</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura fortalecida</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Alerts API y Actions API escuchan en 0.0.0.0:5000/5001, alcanzables directamente desde la red.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Los servicios internos quedan expuestos y se puede saltar Nginx (la frontera de confianza L2 no se cumple).</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>T09 (E); agrava T03, T04, T08</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Bind a 127.0.0.1 en ambos servicios (services/*/app.py) y UFW: deny incoming, allow OpenSSH, allow 80/tcp desde LAB_CIDR (deploy.sh, paso 6). Mitigación M-007.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Nginx :80 es el único punto de entrada; los microservicios solo aceptan conexiones locales.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Implementado en repo; verificado localmente (sockets en 127.0.0.1). Pendiente: desplegar y retest en la VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>G02</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Endpoint /debug/env y app.run(debug=True) en ambos servicios.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Diagnóstico expuesto: variables de entorno del servidor y debugger interactivo de Werkzeug (su PIN se escribe en alerts.log).</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>T06 (I), T10 (E)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Se elimina /debug/env y se ejecuta con debug=False. Mitigación M-008.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Sin superficie de diagnóstico ni debugger interactivo.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Implementado en repo; verificado localmente (GET /debug/env → 404). Pendiente: desplegar y retest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Nginx con banner de versión, sin headers de seguridad y sin denegar rutas ocultas.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Se revela tecnología/versión; faltan X-Content-Type-Options, X-Frame-Options y Referrer-Policy; autoindex no deshabilitado explícitamente.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>T06 (I)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>server_tokens off, tres headers defensivos, autoindex off y location ~ /\. { deny all; } en nginx/lab3-fdsi.conf. Mitigación M-010.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Respuestas sin versión, con headers defensivos y rutas ocultas denegadas.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Implementado en repo. Pendiente: desplegar y retest (curl -I y /.git/config).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>actions-api registra solo remote_addr (127.0.0.1 detrás del proxy) y el campo analyst declarado por el cliente.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Las acciones no tienen origen real y no se pueden vincular 1 a 1 con access.log (WCGW-Assume-1).</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>T05 (R)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>X-Real-IP (que Nginx sobrescribe) se guarda como source_ip en cada acción y se registra en los logs de ambos servicios. Mitigación M-009.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Cada acción queda ligada a IP de origen y timestamp, correlacionable con access.log.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Implementado en repo; verificado localmente (source_ip presente en la respuesta).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Tráfico HTTP sin TLS.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Contenido y rutas visibles en tránsito.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>T04 (T); Information Disclosure en tránsito</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>No implementada en esta iteración (M-002).</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente: TLS 1.2+/1.3 terminado en Nginx, redirect 80 → 443.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Riesgo abierto (Lab 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sin autenticación ni autorización en ningún endpoint.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Cualquier cliente registra o cierra acciones y suplanta analistas.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>T02 (S), T03 (S), T08 (E)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>No implementada en esta iteración (M-001, M-006).</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente: identidad, sesiones y RBAC.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Riesgo abierto (Lab 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Servidor de desarrollo de Flask sin límite de tasa ni de tamaño de payload.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Crecimiento no acotado de ALERTS/ACTIONS y saturación por ráfagas.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>T07 (D)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>No implementada en esta iteración (M-005).</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente: gunicorn y limit_req / client_max_body_size en Nginx.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Riesgo abierto (Lab 4/5).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(threat-model): record verified status per threat, real T01 from the PCAP, TLS plan and cleaned template leftovers
</commit_message>
<xml_diff>
--- a/threat-model/threat-model.xlsx
+++ b/threat-model/threat-model.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Los servicios de Azure en este diagrama se encuentran en la misma región</t>
+          <t>El atacante tiene acceso de red al segmento del laboratorio (LAB_CIDR 192.168.17.0/24) y puede capturar tráfico HTTP en texto claro.</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Los servicios de Azure en este diagrama se encuentran en la misma cuenta de AWS.</t>
+          <t>Las versiones reportadas por Nmap (nginx 1.28.3; Werkzeug 3.1.8 / Python 3.14.4) son las desplegadas, y no hay WAF ni IDS en línea.</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E12"/>
+  <dimension ref="B2:F12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1"/>
   <cols>
     <col width="3.5546875" customWidth="1" min="1" max="1"/>
@@ -733,7 +733,7 @@
     <col width="146.44140625" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="12.77734375" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="9" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="9.109375" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
     <col hidden="1" width="9.109375" customWidth="1" min="7" max="16384"/>
   </cols>
   <sheetData>
@@ -758,6 +758,11 @@
           <t>STRIDE</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
@@ -767,11 +772,24 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>[fuente de la amenaza] [requisitos previos] puede [acción de la amenaza], lo que conduce a [impacto de la amenaza] y afecta negativamente a [activos afectados]</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
+          <t>Un atacante con acceso a la red del laboratorio puede capturar el tráfico HTTP en texto claro (rutas, cabeceras y el cuerpo JSON de las alertas), lo que conduce a la divulgación de las alertas y afecta negativamente a la confidencialidad de los datos de alertas (ALERTS).</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Cliente → Nginx :80 (flujo HTTP sin TLS)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente Lab 4 — TLS. Evidencia: evidence/blue/lab3-http.pcap</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="55.2" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
@@ -794,6 +812,11 @@
           <t>S</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente Lab 4 — identidad. La IP de origen ya queda en los logs</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
@@ -816,6 +839,11 @@
           <t>S</t>
         </is>
       </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente Lab 4 — autenticación de analistas</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -838,6 +866,11 @@
           <t>T</t>
         </is>
       </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente Lab 4 — validación de esquema y TLS</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -860,6 +893,11 @@
           <t>R</t>
         </is>
       </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Mitigado parcialmente — source_ip y X-Real-IP en logs (verificación en la VM pendiente); identidad en Lab 4</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
@@ -882,6 +920,11 @@
           <t>I</t>
         </is>
       </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Corregido — /debug/env eliminado y server_tokens off. Evidencia: evidence/retest/</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
@@ -904,6 +947,11 @@
           <t>D</t>
         </is>
       </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente Lab 4/5 — gunicorn y limit_req</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
@@ -926,6 +974,11 @@
           <t>E</t>
         </is>
       </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente Lab 4 — RBAC</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
@@ -948,6 +1001,11 @@
           <t>E</t>
         </is>
       </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Corregido — puertos 5000/5001 filtered. Evidencia: evidence/retest/nmap_final_after_fix.nmap</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
@@ -968,6 +1026,11 @@
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>E</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Corregido — debug=False y servicios solo en 127.0.0.1. Evidencia: evidence/retest/</t>
         </is>
       </c>
     </row>
@@ -1035,12 +1098,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Validación de esquema de entrada (severity/host/ioc) en alerts-api, más HTTPS/TLS en Lab 4.</t>
+          <t>Validación de esquema de entrada (severity/host/ioc) en alerts-api, más HTTPS/TLS en Lab 4 (TLS 1.2 como mínimo, 1.3 preferido).</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T04, T01</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1183,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[Implementada en repo] Enlazar alerts-api y actions-api únicamente a 127.0.0.1 y configurar UFW (deny incoming; allow OpenSSH; allow 80/tcp desde LAB_CIDR), de modo que Nginx sea el único punto de entrada.</t>
+          <t>[Implementada y verificada en la VM] Enlazar alerts-api y actions-api únicamente a 127.0.0.1 y configurar UFW (deny incoming; allow OpenSSH; allow 80/tcp desde LAB_CIDR), de modo que Nginx sea el único punto de entrada.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1137,7 +1200,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>[Implementada en repo] Ejecutar ambos servicios con debug=False y eliminar el endpoint /debug/env (retira el debugger de Werkzeug y la exposición de variables de entorno).</t>
+          <t>[Implementada y verificada en la VM] Ejecutar ambos servicios con debug=False y eliminar el endpoint /debug/env (retira el debugger de Werkzeug y la exposición de variables de entorno).</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1154,7 +1217,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[Implementada en repo] Registrar la IP real del cliente (X-Real-IP inyectado por Nginx) como source_ip en cada acción y en los logs de ambos servicios, para correlacionarla con access.log.</t>
+          <t>[Implementada en repo; verificación en la VM pendiente] Registrar la IP real del cliente (X-Real-IP inyectado por Nginx) como source_ip en cada acción y en los logs de ambos servicios, para correlacionarla con access.log.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1171,7 +1234,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>[Implementada en repo] Hardening de Nginx: server_tokens off, X-Content-Type-Options, X-Frame-Options, Referrer-Policy, autoindex off y denegación de rutas ocultas.</t>
+          <t>[Implementada y verificada en la VM] Hardening de Nginx: server_tokens off, X-Content-Type-Options, X-Frame-Options, Referrer-Policy, autoindex off y denegación de rutas ocultas.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1391,7 +1454,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Implementado en repo; verificado localmente (sockets en 127.0.0.1). Pendiente: desplegar y retest en la VM.</t>
+          <t>Implementado y verificado en la VM: nmap 5000/5001 pasan de open a filtered (evidence/retest/nmap_final_after_fix.nmap).</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1491,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Implementado en repo; verificado localmente (GET /debug/env → 404). Pendiente: desplegar y retest.</t>
+          <t>Implementado y verificado: GET directo a :5000/debug/env → conexión rechazada (evidence/retest/comparacion-antes-despues.md).</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1528,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Implementado en repo. Pendiente: desplegar y retest (curl -I y /.git/config).</t>
+          <t>Implementado y verificado en la VM: headers presentes, Server sin versión, /.git/config → 403 (evidence/retest/headers_after.txt y hidden_path.txt).</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1565,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Implementado en repo; verificado localmente (source_ip presente en la respuesta).</t>
+          <t>Implementado en repo; verificado localmente. Pendiente: prueba en la VM (POST a /api/actions/actions con source_ip en la respuesta y en access.log).</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1592,12 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>No implementada en esta iteración (M-002).</t>
+          <t>No implementada en Lab 3 (la guía reserva HTTPS al Lab 4). Plan de migración: certificado (autofirmado en el laboratorio), TLS 1.2 como mínimo y 1.3 preferido, suites modernas con forward secrecy, redirect 80 → 443, HSTS una vez estable HTTPS y UFW abriendo 443. Mitigación M-002.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Pendiente: TLS 1.2+/1.3 terminado en Nginx, redirect 80 → 443.</t>
+          <t>Pendiente: Nginx termina TLS 1.2/1.3 en :443 y :80 solo redirige.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: mark T05/M-009/G04 as verified on the VM and move source_ip evidence to evidence/retest
</commit_message>
<xml_diff>
--- a/threat-model/threat-model.xlsx
+++ b/threat-model/threat-model.xlsx
@@ -895,7 +895,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Mitigado parcialmente — source_ip y X-Real-IP en logs (verificación en la VM pendiente); identidad en Lab 4</t>
+          <t>Mitigado y verificado — source_ip y X-Real-IP coinciden en la respuesta, access.log y actions.log (evidence/retest/source_ip_vm.md, 2026-10-16); la identidad autenticada queda para Lab 4</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[Implementada en repo; verificación en la VM pendiente] Registrar la IP real del cliente (X-Real-IP inyectado por Nginx) como source_ip en cada acción y en los logs de ambos servicios, para correlacionarla con access.log.</t>
+          <t>[Implementada y verificada en la VM] Registrar la IP real del cliente (X-Real-IP inyectado por Nginx) como source_ip en cada acción y en los logs de ambos servicios, para correlacionarla con access.log.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Implementado en repo; verificado localmente. Pendiente: prueba en la VM (POST a /api/actions/actions con source_ip en la respuesta y en access.log).</t>
+          <t>Implementado y verificado en la VM (2026-10-16): la IP 192.168.17.130 aparece igual en la respuesta, access.log y actions.log (evidence/retest/source_ip_vm.md).</t>
         </is>
       </c>
     </row>

</xml_diff>